<commit_message>
feat: add 5 interpretation questions focused on SV
</commit_message>
<xml_diff>
--- a/questions/解釈/基本セット/questions.xlsx
+++ b/questions/解釈/基本セット/questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O8"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -555,9 +555,244 @@
         <v>A</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>S03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SVの発見</v>
+      </c>
+      <c r="C4" t="str">
+        <v>The boy playing tennis in the park is my brother.</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>playing...parkがThe boyを修飾していることを見抜く|文全体の主語(S)がThe boy、動詞(V)がisであることを把握する</v>
+      </c>
+      <c r="J4" t="str">
+        <v>S03 解答例 ▷ 分詞による後置修飾</v>
+      </c>
+      <c r="K4" t="str">
+        <v>playing tennis in the parkという現在分詞句が、直前の名詞The boyを修飾しています。文の主語はThe boy、述語動詞はisです。</v>
+      </c>
+      <c r="L4" t="str">
+        <v>playing: 〜している | in the park: 公園で</v>
+      </c>
+      <c r="M4" t="str">
+        <v>公園でテニスをしている少年は私の兄（または弟）です。</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>S04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SVの発見</v>
+      </c>
+      <c r="C5" t="str">
+        <v>To master a foreign language requires a lot of patience.</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>To master...languageという不定詞の名詞用法が文の主語(S)であることを見抜く|requiresが述語動詞(V)であるとわかること</v>
+      </c>
+      <c r="J5" t="str">
+        <v>S04 解答例 ▷ 不定詞の名詞用法</v>
+      </c>
+      <c r="K5" t="str">
+        <v>To master a foreign languageという不定詞のカタマリが文全体の主語になっています。述語動詞はrequiresです。</v>
+      </c>
+      <c r="L5" t="str">
+        <v>master: 習得する | foreign language: 外国語 | require: 必要とする | patience: 忍耐</v>
+      </c>
+      <c r="M5" t="str">
+        <v>外国語を習得することは、多くの忍耐を必要とする。</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v>B</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>S05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SVの発見</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Whether we will go on a picnic tomorrow depends on the weather.</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Whetherが導く名詞節が文全体の主語(S)になっていることを見抜く|depends onが述語動詞(V)であるとわかること</v>
+      </c>
+      <c r="J6" t="str">
+        <v>S05 解答例 ▷ 名詞節（Whether）の主語</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Whether ... tomorrow（明日ピクニックに行くかどうか）という名詞節が文の主語になっています。述語動詞はdependsです。</v>
+      </c>
+      <c r="L6" t="str">
+        <v>whether: 〜するかどうか | go on a picnic: ピクニックに行く | depend on: 〜次第である</v>
+      </c>
+      <c r="M6" t="str">
+        <v>明日ピクニックに行くかどうかは、天気次第です。</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>S06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SVの発見</v>
+      </c>
+      <c r="C7" t="str">
+        <v>The fact that he didn't tell the truth made her angry.</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>that節がThe factと同格であることを理解する|文全体の主語(S)がThe fact、動詞(V)がmadeであることを見抜く</v>
+      </c>
+      <c r="J7" t="str">
+        <v>S06 解答例 ▷ 同格のthatと第5文型</v>
+      </c>
+      <c r="K7" t="str">
+        <v>that he didn't tell the truthはThe factの内容を説明する「同格」のthat節です。主語The factがmade(V) her(O) angry(C)という第5文型を作っています。</v>
+      </c>
+      <c r="L7" t="str">
+        <v>fact: 事実 | truth: 真実 | make O C: OをCにする | angry: 怒って</v>
+      </c>
+      <c r="M7" t="str">
+        <v>彼が真実を言わなかったという事実が、彼女を怒らせた。</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>S07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SVの発見</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Not only the students but also the teacher was surprised at the news.</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Not only A but also Bの構文を見抜く|主語がthe teacherとなり、動詞がwasと単数呼応していることを把握する</v>
+      </c>
+      <c r="J8" t="str">
+        <v>S07 解答例 ▷ 相関接続詞と主語の呼応</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Not only A but also B「AだけでなくBも」の構文では、動詞はBの数に一致します。ここではBがthe teacher(単数)なので、動詞はwereではなくwasになります。</v>
+      </c>
+      <c r="L8" t="str">
+        <v>not only A but also B: AだけでなくBも | surprised at: 〜に驚く | news: 知らせ</v>
+      </c>
+      <c r="M8" t="str">
+        <v>生徒たちだけでなく、その先生もその知らせに驚いた。</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v>B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>